<commit_message>
Remove placeholder Real Estate Agency default values
</commit_message>
<xml_diff>
--- a/public/Cleaned_HandyMap_Jobs.xlsx
+++ b/public/Cleaned_HandyMap_Jobs.xlsx
@@ -506,7 +506,7 @@
 Garage wooden door getting damage with rain waters</v>
       </c>
       <c r="K2" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L2" t="str">
         <v>Aman</v>
@@ -559,7 +559,7 @@
         <v>- Cavity door 820x2340x35</v>
       </c>
       <c r="K3" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L3" t="str">
         <v>Makayla</v>
@@ -612,7 +612,7 @@
         <v>- Garage door is stucking in the middle when they open the door or close it and that time the light is also blinking.</v>
       </c>
       <c r="K4" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L4" t="str">
         <v>Ayesha</v>
@@ -667,7 +667,7 @@
 - Rangehood Replacement</v>
       </c>
       <c r="K5" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L5" t="str">
         <v>Dipali</v>
@@ -723,7 +723,7 @@
 - Master bedroom blinds: as shown in the video the blinds do not stop going down unless we use a clamp on the strings or it hits the ground.</v>
       </c>
       <c r="K6" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L6" t="str">
         <v>Makayla</v>
@@ -778,7 +778,7 @@
 - Bedroom Door not closing</v>
       </c>
       <c r="K7" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L7" t="str">
         <v>Makayla</v>
@@ -834,7 +834,7 @@
 - Latch is not working from entrance to kitchen door</v>
       </c>
       <c r="K8" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L8" t="str">
         <v>Makayla</v>
@@ -892,7 +892,7 @@
 Main Bathroom: Towel rail is loose.</v>
       </c>
       <c r="K9" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L9" t="str">
         <v>Moksh</v>
@@ -945,7 +945,7 @@
         <v>– Cabinet door under the sink has come off</v>
       </c>
       <c r="K10" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L10" t="str">
         <v>Amare</v>
@@ -1001,7 +1001,7 @@
 855W x 2000D</v>
       </c>
       <c r="K11" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L11" t="str">
         <v>Amare</v>
@@ -1054,7 +1054,7 @@
         <v>- Backyard fence needs to get fixed</v>
       </c>
       <c r="K12" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L12" t="str">
         <v>Aman</v>
@@ -1108,7 +1108,7 @@
 - Door lock replaced</v>
       </c>
       <c r="K13" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L13" t="str">
         <v>Jaslin</v>
@@ -1163,7 +1163,7 @@
 3.Flyscreen request – We had previously requested a screen for the living room door. Without it, we are unable to keep the door open as insects and flies enter the house. Kindly arrange installation of a suitable screen.</v>
       </c>
       <c r="K14" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L14" t="str">
         <v>Parneet</v>
@@ -1221,7 +1221,7 @@
 - Main door lock – The door opens randomly.</v>
       </c>
       <c r="K15" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L15" t="str">
         <v>Parneet</v>
@@ -1275,7 +1275,7 @@
 - Mold in living room</v>
       </c>
       <c r="K16" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L16" t="str">
         <v>Mehreen</v>
@@ -1329,7 +1329,7 @@
 - The renters advised that the garden bed timber is becoming loose, resulting in sand falling through. (Backyard)</v>
       </c>
       <c r="K17" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L17" t="str">
         <v>Aman</v>
@@ -1384,7 +1384,7 @@
 - Heating</v>
       </c>
       <c r="K18" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L18" t="str">
         <v>Aman</v>
@@ -1445,7 +1445,7 @@
 - Dry wall plaster damaged repair</v>
       </c>
       <c r="K19" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L19" t="str">
         <v>Ayesha</v>
@@ -1498,7 +1498,7 @@
         <v>- Kitchen tap is wobbly it's need fixing.</v>
       </c>
       <c r="K20" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L20" t="str">
         <v>Prerna</v>
@@ -1554,7 +1554,7 @@
 - Rangehood fan not working</v>
       </c>
       <c r="K21" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L21" t="str">
         <v>Ekta</v>
@@ -1607,7 +1607,7 @@
         <v>- Blind chain got broken</v>
       </c>
       <c r="K22" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L22" t="str">
         <v>Prerna</v>
@@ -1660,7 +1660,7 @@
         <v>- Supply and install new 90cm canopy exhaust fan</v>
       </c>
       <c r="K23" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L23" t="str">
         <v>Aman</v>
@@ -1715,7 +1715,7 @@
 - One electrical switch cover is missing.</v>
       </c>
       <c r="K24" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L24" t="str">
         <v>Ekta</v>
@@ -1768,7 +1768,7 @@
         <v>- Ceiling in lounge area is leaking and has water spots.</v>
       </c>
       <c r="K25" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L25" t="str">
         <v>Ekta</v>
@@ -1821,7 +1821,7 @@
         <v>- Multiple issues please check with tenants</v>
       </c>
       <c r="K26" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L26" t="str">
         <v>Ayesha</v>
@@ -1876,7 +1876,7 @@
 3. One of the Kitchen Island’s cupboard door not closing properly.</v>
       </c>
       <c r="K27" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L27" t="str">
         <v>Mikaela</v>
@@ -1929,7 +1929,7 @@
         <v>- Kitchen - there is also a hole in the pantry, from which rats are entering inside the kitchen.</v>
       </c>
       <c r="K28" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L28" t="str">
         <v>Mikaela</v>
@@ -1982,7 +1982,7 @@
         <v>- Quote to replace roller blinds for full house</v>
       </c>
       <c r="K29" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L29" t="str">
         <v>Mikael</v>
@@ -2037,7 +2037,7 @@
 - The main entrance door squeaks loudly when opening and closing</v>
       </c>
       <c r="K30" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L30" t="str">
         <v>Nadeesha</v>
@@ -2094,7 +2094,7 @@
 - Leak in the kitchen cabinet</v>
       </c>
       <c r="K31" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L31" t="str">
         <v>Dipali</v>
@@ -2148,7 +2148,7 @@
 This appears to be due to missing, damaged, or deteriorated silicone sealing along the base of the shower screens.</v>
       </c>
       <c r="K32" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L32" t="str">
         <v>Ekta</v>
@@ -2201,7 +2201,7 @@
         <v>- Install hooks throughout the house on blinds</v>
       </c>
       <c r="K33" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L33" t="str">
         <v>Dipali</v>
@@ -2255,7 +2255,7 @@
 - Renter has reported that the kitchen sink pipe is leaking. Plumber is required.</v>
       </c>
       <c r="K34" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L34" t="str">
         <v>Ekta</v>
@@ -2308,7 +2308,7 @@
         <v>- The pipe underneath toilet is leaking</v>
       </c>
       <c r="K35" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L35" t="str">
         <v>Parneet</v>
@@ -2363,7 +2363,7 @@
 - Garage remote is also not working</v>
       </c>
       <c r="K36" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L36" t="str">
         <v>Kylie</v>
@@ -2419,7 +2419,7 @@
 - Rangehood fan not working</v>
       </c>
       <c r="K37" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L37" t="str">
         <v>Ekta</v>
@@ -2475,7 +2475,7 @@
 - Back sliding door lock does not work.</v>
       </c>
       <c r="K38" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L38" t="str">
         <v>Makayla</v>
@@ -2528,7 +2528,7 @@
         <v>- Heat duct in the master room is loose.</v>
       </c>
       <c r="K39" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L39" t="str">
         <v>Ekta</v>
@@ -2588,7 +2588,7 @@
 6. Front room shower frame is falling apart.</v>
       </c>
       <c r="K40" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L40" t="str">
         <v>Ekta</v>
@@ -2641,7 +2641,7 @@
         <v>- Supply and install new clothsline</v>
       </c>
       <c r="K41" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L41" t="str">
         <v>Ekta</v>
@@ -2695,7 +2695,7 @@
 -The garage door is occasionally getting stuck when opening.</v>
       </c>
       <c r="K42" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L42" t="str">
         <v>Ekta</v>
@@ -2748,7 +2748,7 @@
         <v>- Fan light needs repalcement</v>
       </c>
       <c r="K43" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L43" t="str">
         <v>Ekta</v>
@@ -2801,7 +2801,7 @@
         <v>- Plaster required on water damage</v>
       </c>
       <c r="K44" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L44" t="str">
         <v>Mehreen</v>
@@ -2857,7 +2857,7 @@
 - Exhaust system issue the buttons does not work</v>
       </c>
       <c r="K45" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L45" t="str">
         <v>Prerna</v>
@@ -2914,7 +2914,7 @@
 - Ensuite RHS sink leaking underneath cupboards</v>
       </c>
       <c r="K46" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L46" t="str">
         <v>Ekta</v>
@@ -2970,7 +2970,7 @@
 - Moisture behind shower wall</v>
       </c>
       <c r="K47" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L47" t="str">
         <v>Makayla</v>
@@ -3023,7 +3023,7 @@
         <v>- Measurements for an upstairs windows where blinds are missing</v>
       </c>
       <c r="K48" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L48" t="str">
         <v>Makayla</v>
@@ -3076,7 +3076,7 @@
         <v>- Tenants are requesting for repair of window screens and locks, which are broken or loose. This is a safety concern, as the back windows could be easily opened, especially given the recent increase in burglaries in the area.</v>
       </c>
       <c r="K49" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L49" t="str">
         <v>Mehreen</v>
@@ -3129,7 +3129,7 @@
         <v>- Regrout the bathroom</v>
       </c>
       <c r="K50" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L50" t="str">
         <v>Ekta</v>
@@ -3186,7 +3186,7 @@
 5. Kitchen gas turns off automatically while using.</v>
       </c>
       <c r="K51" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L51" t="str">
         <v>Ekta</v>
@@ -3239,7 +3239,7 @@
         <v>- Install 2x blind cord anchors / cleats to secure loosely hanging blind cords.</v>
       </c>
       <c r="K52" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L52" t="str">
         <v>Raghav</v>
@@ -3292,7 +3292,7 @@
         <v>- The water is coming from the back garage wooden door when rains</v>
       </c>
       <c r="K53" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L53" t="str">
         <v>Raghav</v>
@@ -3346,7 +3346,7 @@
 - Ac unit leaking</v>
       </c>
       <c r="K54" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L54" t="str">
         <v>Makayla</v>
@@ -3402,7 +3402,7 @@
 – Backyard security screen wheel</v>
       </c>
       <c r="K55" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L55" t="str">
         <v>Ekta</v>
@@ -3456,7 +3456,7 @@
 - Lock on the rear glass is also faulty</v>
       </c>
       <c r="K56" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L56" t="str">
         <v>Ekta</v>
@@ -3509,7 +3509,7 @@
         <v>Check quote for list of work</v>
       </c>
       <c r="K57" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L57" t="str">
         <v>Pankti</v>
@@ -3567,7 +3567,7 @@
 - Door needs to be installed where missing and locks and handle also requote throughout</v>
       </c>
       <c r="K58" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L58" t="str">
         <v>Dipali</v>
@@ -3622,7 +3622,7 @@
 - Towel rail to be repaired/replaced as it has come away</v>
       </c>
       <c r="K59" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L59" t="str">
         <v>Ekta</v>
@@ -3676,7 +3676,7 @@
 - 2090 - Towel rail installation</v>
       </c>
       <c r="K60" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L60" t="str">
         <v>Ekta</v>
@@ -3737,7 +3737,7 @@
 - the ceiling in one corner of Bedroom 2 (the handle of which came off). It also has moisture</v>
       </c>
       <c r="K61" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L61" t="str">
         <v>Ekta</v>
@@ -3791,7 +3791,7 @@
 - Main Bathroom - The renters advised the door knob has been removed as the door was not able to be opened from the inside.</v>
       </c>
       <c r="K62" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L62" t="str">
         <v>Raghav</v>
@@ -3844,7 +3844,7 @@
         <v>The towel rack in the ensuite is broken , not able to hang towels</v>
       </c>
       <c r="K63" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L63" t="str">
         <v>Mounika</v>
@@ -3897,7 +3897,7 @@
         <v>- Inspect leaning rear fence, investigate and advise on the likely cause of the fence leaning, provide supporting photos, and provide a separate quote for the removal and disposal of the internal/non-boundary fence shown in the attached photo.</v>
       </c>
       <c r="K64" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L64" t="str">
         <v>Ekta</v>
@@ -3955,7 +3955,7 @@
 - 1 x Entrance set</v>
       </c>
       <c r="K65" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L65" t="str">
         <v>Makayla</v>
@@ -4009,7 +4009,7 @@
 - Blind hooks for venetian blinds need to be installed and broken blind hooks need replacement on some windows.</v>
       </c>
       <c r="K66" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L66" t="str">
         <v>Rav</v>
@@ -4062,7 +4062,7 @@
         <v>- Entrance Hall - The renters advised that a gap is developing between the tiled floor and the door.</v>
       </c>
       <c r="K67" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L67" t="str">
         <v>Mikaela</v>
@@ -4115,7 +4115,7 @@
         <v>- Kitchen sink tap become loose</v>
       </c>
       <c r="K68" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L68" t="str">
         <v>Mikaela</v>
@@ -4168,7 +4168,7 @@
         <v>- Repair the ensuite light switch, as the light does not stay on.</v>
       </c>
       <c r="K69" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L69" t="str">
         <v>Makayla</v>
@@ -4221,7 +4221,7 @@
         <v>- Loud noise coming from Entrance ceiling</v>
       </c>
       <c r="K70" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L70" t="str">
         <v>Aman</v>
@@ -4274,7 +4274,7 @@
         <v>- Washing machine</v>
       </c>
       <c r="K71" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L71" t="str">
         <v>Dipali</v>
@@ -4327,7 +4327,7 @@
         <v>- Laundry glass replacement</v>
       </c>
       <c r="K72" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L72" t="str">
         <v>Mehreen</v>
@@ -4381,7 +4381,7 @@
 - Quote for repair of damaged wardobe rollers</v>
       </c>
       <c r="K73" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L73" t="str">
         <v>Mikaela</v>
@@ -4435,7 +4435,7 @@
 - Back sliding door doesn't close</v>
       </c>
       <c r="K74" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L74" t="str">
         <v>Sazya</v>
@@ -4490,7 +4490,7 @@
 - The laundry door needs repair</v>
       </c>
       <c r="K75" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L75" t="str">
         <v>Sakshai</v>
@@ -4543,7 +4543,7 @@
         <v>- Loud noise coming from Entrance ceiling ($200+GST)</v>
       </c>
       <c r="K76" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L76" t="str">
         <v>Aman</v>
@@ -4596,7 +4596,7 @@
         <v>- Kitchen sink tap come off</v>
       </c>
       <c r="K77" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L77" t="str">
         <v>Mikaela</v>
@@ -4649,7 +4649,7 @@
         <v>- Check with tenants all maintenance issues and proivde qoutation</v>
       </c>
       <c r="K78" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L78" t="str">
         <v>Ayesha</v>
@@ -4708,7 +4708,7 @@
 5. Roof gutter cleaning</v>
       </c>
       <c r="K79" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L79" t="str">
         <v>Mikaela</v>
@@ -4761,7 +4761,7 @@
         <v>- Dishwasher doesn't turn on</v>
       </c>
       <c r="K80" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L80" t="str">
         <v>Makayla</v>
@@ -4815,7 +4815,7 @@
 - The chimney lights are not working. Can you pls provide quote</v>
       </c>
       <c r="K81" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L81" t="str">
         <v>Makayla</v>
@@ -4868,7 +4868,7 @@
         <v>- Garage remote not functioning</v>
       </c>
       <c r="K82" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L82" t="str">
         <v>Parneet</v>
@@ -4921,7 +4921,7 @@
         <v>- Broken Letterbox</v>
       </c>
       <c r="K83" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L83" t="str">
         <v>Laura</v>
@@ -4974,7 +4974,7 @@
         <v>- Check quote</v>
       </c>
       <c r="K84" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L84" t="str">
         <v>Aman</v>
@@ -5034,7 +5034,7 @@
 - Electric oven and Aircon circuits needs to be protected by RCBO'S</v>
       </c>
       <c r="K85" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L85" t="str">
         <v>Sneha</v>
@@ -5094,7 +5094,7 @@
 - Remove existing moldy shower silicon from common bathroom</v>
       </c>
       <c r="K86" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L86" t="str">
         <v>Prerna</v>
@@ -5147,7 +5147,7 @@
         <v>- Supply and install new wireless door bell</v>
       </c>
       <c r="K87" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L87" t="str">
         <v>Sakshi</v>
@@ -5202,7 +5202,7 @@
 - Rangehood light</v>
       </c>
       <c r="K88" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L88" t="str">
         <v>Ayesha</v>
@@ -5255,7 +5255,7 @@
         <v>- Mould and leaking in bathroom and cracks on wall</v>
       </c>
       <c r="K89" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L89" t="str">
         <v>Ayesha</v>
@@ -5311,7 +5311,7 @@
 - Oven handle is loose</v>
       </c>
       <c r="K90" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L90" t="str">
         <v>Rav</v>
@@ -5364,7 +5364,7 @@
         <v>- Windows flyscreen replacement</v>
       </c>
       <c r="K91" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L91" t="str">
         <v>Sneha</v>
@@ -5418,7 +5418,7 @@
 - Light in the kitchen is not working</v>
       </c>
       <c r="K92" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L92" t="str">
         <v>Sneha</v>
@@ -5471,7 +5471,7 @@
         <v>- Hole in kitchen area - mice entering</v>
       </c>
       <c r="K93" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L93" t="str">
         <v>Mikaela</v>
@@ -5524,7 +5524,7 @@
         <v>- The oven Knob is not operating.</v>
       </c>
       <c r="K94" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L94" t="str">
         <v>Sakshai</v>
@@ -5577,7 +5577,7 @@
         <v>- Dishwasher door is not closing</v>
       </c>
       <c r="K95" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L95" t="str">
         <v>Makayla</v>
@@ -5630,7 +5630,7 @@
         <v>- Cooktop &amp; Range Hood whole replacement</v>
       </c>
       <c r="K96" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L96" t="str">
         <v>Sneha</v>
@@ -5684,7 +5684,7 @@
 - Kitchen - The renters advised that the rangehood filter is not working.</v>
       </c>
       <c r="K97" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L97" t="str">
         <v>Dipali</v>
@@ -5737,7 +5737,7 @@
         <v>- Dishwasher not closing</v>
       </c>
       <c r="K98" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L98" t="str">
         <v>Parneet</v>
@@ -5791,7 +5791,7 @@
 - Cooktop burners are also not working</v>
       </c>
       <c r="K99" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L99" t="str">
         <v>Mehreen</v>
@@ -5845,7 +5845,7 @@
 - The backyard screen door is misaligned and requires adjustment</v>
       </c>
       <c r="K100" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L100" t="str">
         <v>Sneha</v>
@@ -5898,7 +5898,7 @@
         <v>- Paint a draw marks</v>
       </c>
       <c r="K101" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L101" t="str">
         <v>Mikaela</v>
@@ -5951,7 +5951,7 @@
         <v>- Ensuite door. its lose from its hinges</v>
       </c>
       <c r="K102" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L102" t="str">
         <v>Mehreen</v>
@@ -6004,7 +6004,7 @@
         <v>- Shower headset issue water is not coming form headset</v>
       </c>
       <c r="K103" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L103" t="str">
         <v>Mehreen</v>
@@ -6057,7 +6057,7 @@
         <v>- oven door is not opening properly and appears to be stuck at approximately a 45-degree angle</v>
       </c>
       <c r="K104" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L104" t="str">
         <v>Mehreen</v>
@@ -6110,7 +6110,7 @@
         <v>- Leakage in the property</v>
       </c>
       <c r="K105" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L105" t="str">
         <v>Mehreen</v>
@@ -6163,7 +6163,7 @@
         <v>- Remove carpets and change to timber or hybrid floor in bedrooms.</v>
       </c>
       <c r="K106" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L106" t="str">
         <v>Ekta</v>
@@ -6216,7 +6216,7 @@
         <v>- Plaster damaged repair in hallway wall and the indoor garage door, which has a gap at the bottom and is slightly difficult to close.</v>
       </c>
       <c r="K107" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L107" t="str">
         <v>Ekta</v>
@@ -6271,7 +6271,7 @@
 3. Dishwasher clip broken.</v>
       </c>
       <c r="K108" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L108" t="str">
         <v>Ekta</v>
@@ -6326,7 +6326,7 @@
 - Assessment of non working Alfresco fan</v>
       </c>
       <c r="K109" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L109" t="str">
         <v>Makayla</v>
@@ -6379,7 +6379,7 @@
         <v>- Toilet tank leakage in the bowl</v>
       </c>
       <c r="K110" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L110" t="str">
         <v>Mehreen</v>
@@ -6432,7 +6432,7 @@
         <v>- Replace the damaged skirting in kitchen area and paint the affected ceiling on kitchen</v>
       </c>
       <c r="K111" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L111" t="str">
         <v>Rav / Dipali</v>
@@ -6485,7 +6485,7 @@
         <v>- Mould/dampness alfresco celling - If &gt;300, please send quote</v>
       </c>
       <c r="K112" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L112" t="str">
         <v>Mikaela</v>
@@ -6538,7 +6538,7 @@
         <v>- Garage roller door is making an unusual noise</v>
       </c>
       <c r="K113" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L113" t="str">
         <v>Aman</v>
@@ -6592,7 +6592,7 @@
 - Blind curtain string needs to be replaced.</v>
       </c>
       <c r="K114" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L114" t="str">
         <v>Ekta</v>
@@ -6645,7 +6645,7 @@
         <v>23 Wood Grove Burnside Victoria 3023</v>
       </c>
       <c r="K115" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L115" t="str">
         <v>Parneet</v>
@@ -6698,7 +6698,7 @@
         <v/>
       </c>
       <c r="K116" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L116" t="str">
         <v/>
@@ -6751,7 +6751,7 @@
         <v/>
       </c>
       <c r="K117" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L117" t="str">
         <v/>
@@ -6804,7 +6804,7 @@
         <v/>
       </c>
       <c r="K118" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L118" t="str">
         <v/>
@@ -6857,7 +6857,7 @@
         <v>- 2 x Garage remote isnt working</v>
       </c>
       <c r="K119" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L119" t="str">
         <v>Sakshai</v>
@@ -6910,7 +6910,7 @@
         <v>- Oven and dishwasher</v>
       </c>
       <c r="K120" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L120" t="str">
         <v>Dipali</v>
@@ -6963,7 +6963,7 @@
         <v>- Inside and outside few lights are not working</v>
       </c>
       <c r="K121" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L121" t="str">
         <v>Sneha</v>
@@ -7017,7 +7017,7 @@
 - Garage remote mounted on the wall is also not working.</v>
       </c>
       <c r="K122" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L122" t="str">
         <v>Sakshi</v>
@@ -7070,7 +7070,7 @@
         <v>- Replace 3 light bulbs - master bedroom , bedroom 2 and kitchen</v>
       </c>
       <c r="K123" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L123" t="str">
         <v>Mehreen</v>
@@ -7125,7 +7125,7 @@
 - Garage remote – We received two garage remotes. One is working, but the other one is not working.</v>
       </c>
       <c r="K124" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L124" t="str">
         <v>Sneha</v>
@@ -7179,7 +7179,7 @@
 - Flyscreen is damage</v>
       </c>
       <c r="K125" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L125" t="str">
         <v>Mehreen</v>
@@ -7232,7 +7232,7 @@
         <v>- Please provide quote for re-silicon for the shower and skirting damage and toilet holder repair</v>
       </c>
       <c r="K126" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L126" t="str">
         <v>Dipali</v>
@@ -7285,7 +7285,7 @@
         <v>Verandah post - Is rotten at the bottom and is not attached to frame</v>
       </c>
       <c r="K127" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L127" t="str">
         <v>Radiya</v>
@@ -7338,7 +7338,7 @@
         <v>- Side door hinge came off due to the winds</v>
       </c>
       <c r="K128" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L128" t="str">
         <v>Mehreen</v>
@@ -7393,7 +7393,7 @@
 - Oven in the kitchen : The fan had been making a ticking sound in the oven and now the fan isn’t working at all and the oven isn’t turning on (I haven’t been able to use the oven to cook)</v>
       </c>
       <c r="K129" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L129" t="str">
         <v>Dipali</v>
@@ -7446,7 +7446,7 @@
         <v>- Water leakage in bathroom from roof Seems like roof is full of water at the moment. need to arrange someone on urgent basis</v>
       </c>
       <c r="K130" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L130" t="str">
         <v>Mehreen</v>
@@ -7500,7 +7500,7 @@
 - One black blind required at the window to help reduce the direct sunlight.</v>
       </c>
       <c r="K131" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L131" t="str">
         <v>Sneha</v>
@@ -7553,7 +7553,7 @@
         <v>- Gas leakage from stove. need to arrange someone to look into this</v>
       </c>
       <c r="K132" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L132" t="str">
         <v>Mehreen</v>
@@ -7606,7 +7606,7 @@
         <v>- Broken blind in the lounge. need to fix/replace it</v>
       </c>
       <c r="K133" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L133" t="str">
         <v>Mehreen</v>
@@ -7660,7 +7660,7 @@
 - The backyard screen door is misaligned and requires adjustment</v>
       </c>
       <c r="K134" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L134" t="str">
         <v>Sneha</v>
@@ -7713,7 +7713,7 @@
         <v>- Both master bathroom and main bathroom shower silicon to be replace.</v>
       </c>
       <c r="K135" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L135" t="str">
         <v>Ekta</v>
@@ -7767,7 +7767,7 @@
 - Turf needs to be fixed.</v>
       </c>
       <c r="K136" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L136" t="str">
         <v>Ekta</v>
@@ -7820,7 +7820,7 @@
         <v>– Garage door not working with switch on the wall or remote</v>
       </c>
       <c r="K137" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L137" t="str">
         <v>Sakshi</v>
@@ -7873,7 +7873,7 @@
         <v>- Tenants have reported a roof leak that is causing mold to form and one light is not working. We need to arrange the handyman to check the inspect the issue and arrange for repairs. Please let us know if you approve this or if you would like us to coordinate with you.</v>
       </c>
       <c r="K138" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L138" t="str">
         <v>Ayesha</v>
@@ -7926,7 +7926,7 @@
         <v>- Toilet door handle is stuck</v>
       </c>
       <c r="K139" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L139" t="str">
         <v>Monika</v>
@@ -7979,7 +7979,7 @@
         <v>The installation of mail Box is required at the property</v>
       </c>
       <c r="K140" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L140" t="str">
         <v>Sakshai</v>
@@ -8032,7 +8032,7 @@
         <v>- Leakage in the property</v>
       </c>
       <c r="K141" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L141" t="str">
         <v>Mehreen</v>
@@ -8085,7 +8085,7 @@
         <v>- Dish washer is not working properly. The dishwasher is not draining properly and dishes come unclean.</v>
       </c>
       <c r="K142" t="str">
-        <v>Ray White / Barry Plant Property Management</v>
+        <v/>
       </c>
       <c r="L142" t="str">
         <v>Sakshai</v>

</xml_diff>